<commit_message>
dataset connnected to sql
</commit_message>
<xml_diff>
--- a/dataset/raw/ecommerce_funnel_raw.xlsx
+++ b/dataset/raw/ecommerce_funnel_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2b71c94e946cc3d6/Documents/Personal Programming Projects/Data-Analyst/E-Commerce-Purchase-Funnel/dataset/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5882468C-B3C6-4875-97FA-D12FE303D6E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{5882468C-B3C6-4875-97FA-D12FE303D6E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F0F138E-FD31-46FA-95AD-AF2F47527021}"/>
   <bookViews>
-    <workbookView xWindow="19875" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{ABEC5AD0-5A71-427B-B1C8-B60C91F769A9}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{ABEC5AD0-5A71-427B-B1C8-B60C91F769A9}"/>
   </bookViews>
   <sheets>
     <sheet name="ecommerce_funnel_raw" sheetId="1" r:id="rId1"/>
@@ -10386,6 +10386,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48012E6B-51C6-4BC5-B368-83FA89F06164}">
   <dimension ref="A1:J1826"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="11.23046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.3046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.69140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.3046875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.53515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.23046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.4609375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A1" t="s">

</xml_diff>